<commit_message>
update 2026-09-27 20:30 (plan 2026-09)
</commit_message>
<xml_diff>
--- a/db2dcd3c52_plan_2026-09.xlsx
+++ b/db2dcd3c52_plan_2026-09.xlsx
@@ -66,7 +66,7 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00C62828"/>
+      <color rgb="002E7D32"/>
       <sz val="11"/>
     </font>
     <font>
@@ -76,11 +76,11 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="002E7D32"/>
+      <color rgb="00C62828"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -100,6 +100,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF0F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDECEA"/>
       </patternFill>
     </fill>
   </fills>
@@ -173,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -226,10 +231,16 @@
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -634,7 +645,7 @@
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>6 يوم = 0.2 شهر</t>
+          <t>259 يوم = 8.5 شهر</t>
         </is>
       </c>
       <c r="E2" s="3" t="n"/>
@@ -1125,7 +1136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1202,17 +1213,17 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>1268</v>
+        <v>5818</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>3150</v>
       </c>
       <c r="D4" s="17" t="n">
-        <v>1881.666666666667</v>
+        <v>-2667.683397683398</v>
       </c>
       <c r="E4" s="18" t="inlineStr">
         <is>
-          <t>زيادة كبيرة - راجعها</t>
+          <t>قصاص كبير - نصايح احتياطية</t>
         </is>
       </c>
     </row>
@@ -1223,17 +1234,17 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>3044</v>
+        <v>1267</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>1050</v>
       </c>
-      <c r="D5" s="19" t="n">
-        <v>-1994</v>
+      <c r="D5" s="17" t="n">
+        <v>-217.4322779922782</v>
       </c>
       <c r="E5" s="18" t="inlineStr">
         <is>
-          <t>قصاص كبير - نصايح احتياطية</t>
+          <t>ناقص شوية - واقعي</t>
         </is>
       </c>
     </row>
@@ -1243,18 +1254,19 @@
           <t>بنزين وصيانة الموتوسيكل</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n">
-        <v>913</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>3300</v>
-      </c>
-      <c r="D6" s="17" t="n">
-        <v>2386.8</v>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>زيادة كبيرة - راجعها</t>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>جديد</t>
         </is>
       </c>
     </row>
@@ -1264,19 +1276,18 @@
           <t>مشتريات ومحلات</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>جديد</t>
+      <c r="B7" s="10" t="n">
+        <v>525</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>1050</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>525.4647366795367</v>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>زيادة كبيرة - راجعها</t>
         </is>
       </c>
     </row>
@@ -1287,13 +1298,13 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>1522</v>
+        <v>5219</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>450</v>
       </c>
-      <c r="D8" s="19" t="n">
-        <v>-1072</v>
+      <c r="D8" s="17" t="n">
+        <v>-4768.926247104248</v>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
@@ -1307,19 +1318,18 @@
           <t>كافيهات وترفيه</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>جديد</t>
+      <c r="B9" s="10" t="n">
+        <v>552</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <v>-401.8454671814671</v>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>قصاص كبير - نصايح احتياطية</t>
         </is>
       </c>
     </row>
@@ -1329,19 +1339,18 @@
           <t>بقالة وسوبر ماركت</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>جديد</t>
+      <c r="B10" s="10" t="n">
+        <v>345</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>600</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>255.1817915057915</v>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>زيادة بسيطة</t>
         </is>
       </c>
     </row>
@@ -1351,19 +1360,18 @@
           <t>صحة وصيدليات</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>جديد</t>
+      <c r="B11" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>450</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>350.1003861003861</v>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>زيادة كبيرة - راجعها</t>
         </is>
       </c>
     </row>
@@ -1373,19 +1381,18 @@
           <t>تسوق أونلاين</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>جديد</t>
+      <c r="B12" s="10" t="n">
+        <v>82</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>220</v>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>138.4055212355212</v>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>زيادة بسيطة</t>
         </is>
       </c>
     </row>
@@ -1417,19 +1424,18 @@
           <t>تحويلات ومدفوعات (أصدقاء)</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>جديد</t>
+      <c r="B14" s="10" t="n">
+        <v>508</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>450</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>-58.26102857142865</v>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>ناقص شوية - واقعي</t>
         </is>
       </c>
     </row>
@@ -1478,21 +1484,42 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>أخرى (غير مصنف) (غير مخطط له)</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="n">
+        <v>1507</v>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>-1507</v>
+      </c>
+      <c r="E17" s="21" t="inlineStr">
+        <is>
+          <t>صنّفه في الخطة القادمة</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n">
-        <v>6748</v>
-      </c>
-      <c r="C17" s="13" t="n">
+      <c r="B18" s="13" t="n">
+        <v>14415</v>
+      </c>
+      <c r="C18" s="13" t="n">
         <v>14990</v>
       </c>
-      <c r="D17" s="13" t="n">
-        <v>8242</v>
-      </c>
-      <c r="E17" s="12" t="inlineStr"/>
+      <c r="D18" s="13" t="n">
+        <v>575</v>
+      </c>
+      <c r="E18" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1559,7 +1586,7 @@
       <c r="C3" s="5" t="n">
         <v>41852.25994355001</v>
       </c>
-      <c r="D3" s="20" t="n">
+      <c r="D3" s="22" t="n">
         <v>958147.74005645</v>
       </c>
     </row>
@@ -1573,7 +1600,7 @@
       <c r="C4" s="5" t="n">
         <v>89012.43401553178</v>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D4" s="22" t="n">
         <v>910987.5659844682</v>
       </c>
     </row>
@@ -1587,7 +1614,7 @@
       <c r="C5" s="5" t="n">
         <v>142153.6985852216</v>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="22" t="n">
         <v>857846.3014147785</v>
       </c>
     </row>
@@ -1601,7 +1628,7 @@
       <c r="C6" s="5" t="n">
         <v>202034.6056352133</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="22" t="n">
         <v>797965.3943647867</v>
       </c>
     </row>
@@ -1615,7 +1642,7 @@
       <c r="C7" s="5" t="n">
         <v>269509.9105261498</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="22" t="n">
         <v>730490.0894738501</v>
       </c>
     </row>
@@ -1629,7 +1656,7 @@
       <c r="C8" s="5" t="n">
         <v>345542.7729930434</v>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D8" s="22" t="n">
         <v>654457.2270069567</v>
       </c>
     </row>
@@ -1643,7 +1670,7 @@
       <c r="C9" s="5" t="n">
         <v>431218.5055333205</v>
       </c>
-      <c r="D9" s="20" t="n">
+      <c r="D9" s="22" t="n">
         <v>568781.4944666794</v>
       </c>
     </row>
@@ -1657,7 +1684,7 @@
       <c r="C10" s="5" t="n">
         <v>527760.065434597</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="22" t="n">
         <v>472239.934565403</v>
       </c>
     </row>
@@ -1671,7 +1698,7 @@
       <c r="C11" s="5" t="n">
         <v>636545.5115793402</v>
       </c>
-      <c r="D11" s="20" t="n">
+      <c r="D11" s="22" t="n">
         <v>363454.4884206598</v>
       </c>
     </row>
@@ -1685,7 +1712,7 @@
       <c r="C12" s="5" t="n">
         <v>759127.6752093101</v>
       </c>
-      <c r="D12" s="20" t="n">
+      <c r="D12" s="22" t="n">
         <v>240872.3247906899</v>
       </c>
     </row>
@@ -1699,7 +1726,7 @@
       <c r="C13" s="5" t="n">
         <v>897256.3254352931</v>
       </c>
-      <c r="D13" s="20" t="n">
+      <c r="D13" s="22" t="n">
         <v>102743.6745647069</v>
       </c>
     </row>
@@ -1713,7 +1740,7 @@
       <c r="C14" s="9" t="n">
         <v>1052903.145888275</v>
       </c>
-      <c r="D14" s="21" t="n">
+      <c r="D14" s="23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1727,7 +1754,7 @@
       <c r="C15" s="9" t="n">
         <v>1228289.879035151</v>
       </c>
-      <c r="D15" s="21" t="n">
+      <c r="D15" s="23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1741,7 +1768,7 @@
       <c r="C16" s="9" t="n">
         <v>1425920.039898128</v>
       </c>
-      <c r="D16" s="21" t="n">
+      <c r="D16" s="23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1755,7 +1782,7 @@
       <c r="C17" s="9" t="n">
         <v>1648614.651867538</v>
       </c>
-      <c r="D17" s="21" t="n">
+      <c r="D17" s="23" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>